<commit_message>
feat: pagination, bulk import
</commit_message>
<xml_diff>
--- a/Client/public/asset-import-template.xlsx
+++ b/Client/public/asset-import-template.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AN1"/>
+  <dimension ref="A1:AO1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -408,134 +408,137 @@
         <v>category_name</v>
       </c>
       <c r="C1" t="str">
+        <v>category_slug</v>
+      </c>
+      <c r="D1" t="str">
         <v>model</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>serial_number</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>location_code</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>location_name</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>purchase_date</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>warranty_expiry</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>status</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>notes</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>activation_date</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>capacity_gb</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>carrier</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>device_type</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>encryption_enabled</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>file_system</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="R1" t="str">
         <v>firmware_version</v>
       </c>
-      <c r="R1" t="str">
+      <c r="S1" t="str">
         <v>generation</v>
       </c>
-      <c r="S1" t="str">
+      <c r="T1" t="str">
         <v>host_name</v>
       </c>
-      <c r="T1" t="str">
+      <c r="U1" t="str">
         <v>imei_1</v>
       </c>
-      <c r="U1" t="str">
+      <c r="V1" t="str">
         <v>imei_2</v>
       </c>
-      <c r="V1" t="str">
+      <c r="W1" t="str">
         <v>ip_address</v>
       </c>
-      <c r="W1" t="str">
+      <c r="X1" t="str">
         <v>mac_lan</v>
       </c>
-      <c r="X1" t="str">
+      <c r="Y1" t="str">
         <v>mac_wifi</v>
       </c>
-      <c r="Y1" t="str">
+      <c r="Z1" t="str">
         <v>monitor_size_inch</v>
       </c>
-      <c r="Z1" t="str">
+      <c r="AA1" t="str">
         <v>os</v>
       </c>
-      <c r="AA1" t="str">
+      <c r="AB1" t="str">
         <v>panel_type</v>
       </c>
-      <c r="AB1" t="str">
+      <c r="AC1" t="str">
         <v>phone_number</v>
       </c>
-      <c r="AC1" t="str">
+      <c r="AD1" t="str">
         <v>plan_name</v>
       </c>
-      <c r="AD1" t="str">
+      <c r="AE1" t="str">
         <v>ports</v>
       </c>
-      <c r="AE1" t="str">
+      <c r="AF1" t="str">
         <v>processor</v>
       </c>
-      <c r="AF1" t="str">
+      <c r="AG1" t="str">
         <v>ram_gb</v>
       </c>
-      <c r="AG1" t="str">
+      <c r="AH1" t="str">
         <v>ram_type</v>
       </c>
-      <c r="AH1" t="str">
+      <c r="AI1" t="str">
         <v>refresh_rate_hz</v>
       </c>
-      <c r="AI1" t="str">
+      <c r="AJ1" t="str">
         <v>resolution</v>
       </c>
-      <c r="AJ1" t="str">
+      <c r="AK1" t="str">
         <v>sim_number</v>
       </c>
-      <c r="AK1" t="str">
+      <c r="AL1" t="str">
         <v>sim_previously_used_by</v>
       </c>
-      <c r="AL1" t="str">
+      <c r="AM1" t="str">
         <v>storage_gb</v>
       </c>
-      <c r="AM1" t="str">
+      <c r="AN1" t="str">
         <v>storage_type</v>
       </c>
-      <c r="AN1" t="str">
+      <c r="AO1" t="str">
         <v>usb_type</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AN1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AO1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Asset bulk import (v1)</v>
+        <v>Asset bulk import (v2)</v>
       </c>
     </row>
     <row r="2">
@@ -550,37 +553,42 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Do not add a category_slug column when importing from the New Asset page (category comes from the UI).</v>
+        <v>Provide category_name or category_slug per row (mixed/predefined/custom categories supported).</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>For multi-category files (advanced), include category_slug as the first column — not used by the current UI flow.</v>
+        <v>If both category_name and category_slug are blank, page-selected category is used as fallback.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Dates: yyyy-mm-dd. Booleans: true/false. Empty or N/A = optional field omitted.</v>
+        <v>For custom fields in custom categories, use columns prefixed with custom_ (example: custom_band, custom_vendor).</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>asset_tag is system-generated; do not add a column for it.</v>
+        <v>Dates: yyyy-mm-dd. Booleans: true/false. Empty or N/A = optional field omitted.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Reject: duplicate (category + serial) within the same file; employee/assignment columns.</v>
+        <v>asset_tag is system-generated; do not add a column for it.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>template_version in app: 1</v>
+        <v>Reject: duplicate serial_number within the same file; employee/assignment columns; unknown random headers.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>template_version in app: 2</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>